<commit_message>
delete post bug fix
</commit_message>
<xml_diff>
--- a/module-wise-test-scenarios-and-cases.xlsx
+++ b/module-wise-test-scenarios-and-cases.xlsx
@@ -663,10 +663,10 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13">
@@ -677,10 +677,10 @@
       </c>
       <c r="B13" s="5" t="inlineStr"/>
       <c r="C13" s="5" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>98</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -7983,7 +7983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8148,423 +8148,393 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>TS-DEL-05</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Delete Post</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Delete API actually removes the post from the database</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Verify that a successful delete is reflected in the listing and detail endpoints, not just in the API response.</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Regression, Critical, Bug-Guard</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Test Cases</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="28" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>Scenario ID</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>Module Name</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>Coverage Type</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>Preconditions</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr">
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr">
+      <c r="J12" s="3" t="inlineStr">
         <is>
           <t>Steps</t>
         </is>
       </c>
-      <c r="K11" s="3" t="inlineStr">
+      <c r="K12" s="3" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>TC-DEL-01</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>TS-DEL-01</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Delete Post</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>Author deletes their own post and is returned to the home page</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>Smoke</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>The user is logged in as the post's author.</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>The author's existing post.</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="J13" s="4" t="inlineStr">
         <is>
           <t>1. Open the post detail page for the author's post.
 2. Click Delete.
 3. Confirm "Delete this post?".</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr">
+      <c r="K13" s="4" t="inlineStr">
         <is>
           <t>The user is returned to the home page. The deleted post no longer appears in the list.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>TC-DEL-02</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>TS-DEL-02</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Delete Post</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Cancelling the confirmation keeps the post intact</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>Regression</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>The user is logged in as the post's author.</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>The author's existing post.</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr">
+      <c r="J14" s="4" t="inlineStr">
         <is>
           <t>1. Open the post detail page.
 2. Click Delete.
 3. Cancel the "Delete this post?" prompt.</t>
         </is>
       </c>
-      <c r="K13" s="4" t="inlineStr">
+      <c r="K14" s="4" t="inlineStr">
         <is>
           <t>The user remains on the post detail page. The post is not deleted and still appears on the home page.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>TC-DEL-03</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>TS-DEL-03</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Delete Post</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>A user cannot delete a post that belongs to someone else</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>Regression</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>User Sara is logged in. The post belongs to Ali Khan.</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="I15" s="4" t="inlineStr">
         <is>
           <t>Other user: sara.n / sara.n@gmail.com
 Post owner: ali.khan</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr">
+      <c r="J15" s="4" t="inlineStr">
         <is>
           <t>1. Log in as Sara.
 2. Try to delete Ali Khan's post.</t>
         </is>
       </c>
-      <c r="K14" s="4" t="inlineStr">
+      <c r="K15" s="4" t="inlineStr">
         <is>
           <t>The action is rejected with the message "You can only delete your own posts". The post still appears on the home page.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>TC-DEL-04</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>TS-DEL-04</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Delete Post</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>Deleting a non-existent post shows a not-found message</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>The user is logged in. The chosen post does not exist.</t>
-        </is>
-      </c>
-      <c r="I15" s="4" t="inlineStr">
-        <is>
-          <t>Post reference: 999999</t>
-        </is>
-      </c>
-      <c r="J15" s="4" t="inlineStr">
-        <is>
-          <t>1. While logged in, try to delete a post that does not exist.</t>
-        </is>
-      </c>
-      <c r="K15" s="4" t="inlineStr">
-        <is>
-          <t>The validation message "Post not found" is displayed and no post is deleted.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
+          <t>TC-DEL-04</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>TS-DEL-04</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Delete Post</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Deleting a non-existent post shows a not-found message</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>The user is logged in. The chosen post does not exist.</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>Post reference: 999999</t>
+        </is>
+      </c>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>1. While logged in, try to delete a post that does not exist.</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>The validation message "Post not found" is displayed and no post is deleted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
           <t>TC-DEL-05</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>TS-DEL-01</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Delete Post</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>Deleting the only existing post shows the empty list message</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>Regression</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr">
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>Edge</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>Only one post exists, owned by the current user.</t>
         </is>
       </c>
-      <c r="I16" s="4" t="inlineStr">
+      <c r="I17" s="4" t="inlineStr">
         <is>
           <t>The user's only post.</t>
         </is>
       </c>
-      <c r="J16" s="4" t="inlineStr">
+      <c r="J17" s="4" t="inlineStr">
         <is>
           <t>1. Open the post detail page.
 2. Click Delete and confirm.</t>
         </is>
       </c>
-      <c r="K16" s="4" t="inlineStr">
+      <c r="K17" s="4" t="inlineStr">
         <is>
           <t>The home page opens and shows "No posts yet. Be the first to write one!".</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>TC-DEL-06</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>TS-DEL-03</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Delete Post</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>A delete attempt without a valid session is rejected</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="H17" s="4" t="inlineStr">
-        <is>
-          <t>The user is not signed in.</t>
-        </is>
-      </c>
-      <c r="I17" s="4" t="inlineStr">
-        <is>
-          <t>An existing post.</t>
-        </is>
-      </c>
-      <c r="J17" s="4" t="inlineStr">
-        <is>
-          <t>1. Without being signed in, try to delete a post.</t>
-        </is>
-      </c>
-      <c r="K17" s="4" t="inlineStr">
-        <is>
-          <t>The action is rejected with the message "Missing token". The post still exists.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>TC-DEL-07</t>
+          <t>TC-DEL-06</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -8579,7 +8549,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>A delete attempt with an invalid session is rejected</t>
+          <t>A delete attempt without a valid session is rejected</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -8599,7 +8569,7 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>The user's session is invalid or has expired.</t>
+          <t>The user is not signed in.</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -8609,57 +8579,114 @@
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>1. With an invalid session, try to delete a post.</t>
+          <t>1. Without being signed in, try to delete a post.</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>The action is rejected with the message "Invalid or expired token". The post still exists.</t>
+          <t>The action is rejected with the message "Missing token". The post still exists.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
+          <t>TC-DEL-07</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>TS-DEL-03</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Delete Post</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>A delete attempt with an invalid session is rejected</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>The user's session is invalid or has expired.</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>An existing post.</t>
+        </is>
+      </c>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>1. With an invalid session, try to delete a post.</t>
+        </is>
+      </c>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>The action is rejected with the message "Invalid or expired token". The post still exists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
           <t>TC-DEL-08</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>TS-DEL-01</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>Delete Post</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>End-to-end: register, publish a post, delete it, and verify it is gone</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>Smoke</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="G20" s="4" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="H20" s="4" t="inlineStr">
         <is>
           <t>A new visitor with no posts.</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr">
+      <c r="I20" s="4" t="inlineStr">
         <is>
           <t>Username: noor.e
 Email: noor.e@gmail.com
@@ -8668,7 +8695,7 @@
 Content: Bye</t>
         </is>
       </c>
-      <c r="J19" s="4" t="inlineStr">
+      <c r="J20" s="4" t="inlineStr">
         <is>
           <t>1. Register a new account.
 2. Create a post with the title and content above.
@@ -8677,15 +8704,189 @@
 5. Try to open the deleted post's detail page again.</t>
         </is>
       </c>
-      <c r="K19" s="4" t="inlineStr">
+      <c r="K20" s="4" t="inlineStr">
         <is>
           <t>The post no longer appears on the home page. Opening the deleted post's detail page shows "Failed to load post: Post not found".</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>TC-DEL-09</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>TS-DEL-05</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Delete Post</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>After a successful delete, the post no longer appears in the public list</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Smoke</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>The user is logged in as the post's author and the post exists.</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>Title: Delete me — bug-guard
+Content: Should be gone after delete.</t>
+        </is>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>1. While logged in, send the delete request for the user's post.
+2. Confirm the request returns a successful response.
+3. Refresh the home page (or fetch the public posts list).</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>The deleted post is not present in the public posts list. The deleted post's detail page shows "Post not found". Notes: this case guards against the regression where the delete API returns OK but the row is never removed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>TC-DEL-10</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>TS-DEL-05</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Delete Post</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>After a successful delete, opening the post directly shows a not-found message</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>The user has just deleted their own post.</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>The deleted post's reference.</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>1. After deleting a post, open its detail page directly using its reference.</t>
+        </is>
+      </c>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>The page shows "Failed to load post: Post not found". The post can no longer be retrieved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>TC-DEL-11</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>TS-DEL-05</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Delete Post</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Re-deleting the same post a second time is rejected as not found</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>The user has already deleted a post.</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>The previously-deleted post's reference.</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>1. Send a second delete request for the same post the user just deleted.</t>
+        </is>
+      </c>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>The second attempt is rejected with the message "Post not found". Notes: protects against the bug where the row was never actually removed, in which case a second delete would still report success.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A10:K10"/>
+    <mergeCell ref="A11:K11"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A3:K3"/>
   </mergeCells>

</xml_diff>